<commit_message>
Minor update to character traits.
</commit_message>
<xml_diff>
--- a/story_simulator/data/character_traits.xlsx
+++ b/story_simulator/data/character_traits.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
   <si>
     <t>Description</t>
   </si>
@@ -630,6 +630,57 @@
   </si>
   <si>
     <t>compassionate</t>
+  </si>
+  <si>
+    <t>confident</t>
+  </si>
+  <si>
+    <t>conscientous</t>
+  </si>
+  <si>
+    <t>considerate</t>
+  </si>
+  <si>
+    <t>courageous</t>
+  </si>
+  <si>
+    <t>courteous</t>
+  </si>
+  <si>
+    <t>creative</t>
+  </si>
+  <si>
+    <t>curious</t>
+  </si>
+  <si>
+    <t>daring</t>
+  </si>
+  <si>
+    <t>decent</t>
+  </si>
+  <si>
+    <t>decisive</t>
+  </si>
+  <si>
+    <t>educated</t>
+  </si>
+  <si>
+    <t>dependable</t>
+  </si>
+  <si>
+    <t>determined</t>
+  </si>
+  <si>
+    <t>dignified</t>
+  </si>
+  <si>
+    <t>diligent</t>
+  </si>
+  <si>
+    <t>diplomatic</t>
+  </si>
+  <si>
+    <t>disciplined</t>
   </si>
 </sst>
 </file>
@@ -950,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C199"/>
+  <dimension ref="A1:C216"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -2555,6 +2606,142 @@
         <v>1</v>
       </c>
     </row>
+    <row r="200" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B200" t="s">
+        <v>201</v>
+      </c>
+      <c r="C200" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B201" t="s">
+        <v>202</v>
+      </c>
+      <c r="C201" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B202" t="s">
+        <v>203</v>
+      </c>
+      <c r="C202" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B203" t="s">
+        <v>204</v>
+      </c>
+      <c r="C203" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B204" t="s">
+        <v>205</v>
+      </c>
+      <c r="C204" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="205" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B205" t="s">
+        <v>206</v>
+      </c>
+      <c r="C205" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B206" t="s">
+        <v>207</v>
+      </c>
+      <c r="C206" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B207" t="s">
+        <v>208</v>
+      </c>
+      <c r="C207" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="208" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B208" t="s">
+        <v>209</v>
+      </c>
+      <c r="C208" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="209" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B209" t="s">
+        <v>210</v>
+      </c>
+      <c r="C209" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B210" t="s">
+        <v>211</v>
+      </c>
+      <c r="C210" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B211" t="s">
+        <v>212</v>
+      </c>
+      <c r="C211" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B212" t="s">
+        <v>213</v>
+      </c>
+      <c r="C212" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B213" t="s">
+        <v>214</v>
+      </c>
+      <c r="C213" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="214" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B214" t="s">
+        <v>215</v>
+      </c>
+      <c r="C214" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B215" t="s">
+        <v>216</v>
+      </c>
+      <c r="C215" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B216" t="s">
+        <v>217</v>
+      </c>
+      <c r="C216" s="1">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added some more character traits. Doing things bit by bit.
</commit_message>
<xml_diff>
--- a/story_simulator/data/character_traits.xlsx
+++ b/story_simulator/data/character_traits.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
   <si>
     <t>Description</t>
   </si>
@@ -681,6 +681,105 @@
   </si>
   <si>
     <t>disciplined</t>
+  </si>
+  <si>
+    <t>discreet</t>
+  </si>
+  <si>
+    <t>dynamic</t>
+  </si>
+  <si>
+    <t>easy-going</t>
+  </si>
+  <si>
+    <t>efficient</t>
+  </si>
+  <si>
+    <t>eloquent</t>
+  </si>
+  <si>
+    <t>empathetic</t>
+  </si>
+  <si>
+    <t>encouraging</t>
+  </si>
+  <si>
+    <t>energetic</t>
+  </si>
+  <si>
+    <t>enthusiastic</t>
+  </si>
+  <si>
+    <t>exuberant</t>
+  </si>
+  <si>
+    <t>fair</t>
+  </si>
+  <si>
+    <t>faithful</t>
+  </si>
+  <si>
+    <t>fearless</t>
+  </si>
+  <si>
+    <t>firm</t>
+  </si>
+  <si>
+    <t>flexible</t>
+  </si>
+  <si>
+    <t>focused</t>
+  </si>
+  <si>
+    <t>forgiving</t>
+  </si>
+  <si>
+    <t>frank</t>
+  </si>
+  <si>
+    <t>funny</t>
+  </si>
+  <si>
+    <t>generous</t>
+  </si>
+  <si>
+    <t>gentle</t>
+  </si>
+  <si>
+    <t>genuine</t>
+  </si>
+  <si>
+    <t>gracious</t>
+  </si>
+  <si>
+    <t>gregarious</t>
+  </si>
+  <si>
+    <t>hard-working</t>
+  </si>
+  <si>
+    <t>helpful</t>
+  </si>
+  <si>
+    <t>honest</t>
+  </si>
+  <si>
+    <t>humble</t>
+  </si>
+  <si>
+    <t>humorous</t>
+  </si>
+  <si>
+    <t>idealistic</t>
+  </si>
+  <si>
+    <t>imaginative</t>
+  </si>
+  <si>
+    <t>impartial</t>
+  </si>
+  <si>
+    <t>incisive</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C216"/>
+  <dimension ref="A1:C249"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -2688,7 +2787,7 @@
     </row>
     <row r="210" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B210" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C210" s="1">
         <v>1</v>
@@ -2696,7 +2795,7 @@
     </row>
     <row r="211" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B211" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C211" s="1">
         <v>1</v>
@@ -2704,23 +2803,23 @@
     </row>
     <row r="212" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B212" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C212" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="213" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B213" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C213" s="1">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B214" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C214" s="1">
         <v>1</v>
@@ -2728,7 +2827,7 @@
     </row>
     <row r="215" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B215" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C215" s="1">
         <v>1</v>
@@ -2736,9 +2835,273 @@
     </row>
     <row r="216" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B216" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C216" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B217" t="s">
+        <v>219</v>
+      </c>
+      <c r="C217" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B218" t="s">
+        <v>220</v>
+      </c>
+      <c r="C218" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="219" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B219" t="s">
+        <v>211</v>
+      </c>
+      <c r="C219" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B220" t="s">
+        <v>221</v>
+      </c>
+      <c r="C220" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="221" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B221" t="s">
+        <v>222</v>
+      </c>
+      <c r="C221" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B222" t="s">
+        <v>223</v>
+      </c>
+      <c r="C222" s="1">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="223" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B223" t="s">
+        <v>224</v>
+      </c>
+      <c r="C223" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B224" t="s">
+        <v>225</v>
+      </c>
+      <c r="C224" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="225" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B225" t="s">
+        <v>226</v>
+      </c>
+      <c r="C225" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B226" t="s">
+        <v>227</v>
+      </c>
+      <c r="C226" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="227" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B227" t="s">
+        <v>228</v>
+      </c>
+      <c r="C227" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B228" t="s">
+        <v>229</v>
+      </c>
+      <c r="C228" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B229" t="s">
+        <v>230</v>
+      </c>
+      <c r="C229" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="230" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B230" t="s">
+        <v>231</v>
+      </c>
+      <c r="C230" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B231" t="s">
+        <v>232</v>
+      </c>
+      <c r="C231" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B232" t="s">
+        <v>233</v>
+      </c>
+      <c r="C232" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B233" t="s">
+        <v>234</v>
+      </c>
+      <c r="C233" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="234" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B234" t="s">
+        <v>235</v>
+      </c>
+      <c r="C234" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="235" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B235" t="s">
+        <v>236</v>
+      </c>
+      <c r="C235" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="236" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B236" t="s">
+        <v>237</v>
+      </c>
+      <c r="C236" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="237" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B237" t="s">
+        <v>238</v>
+      </c>
+      <c r="C237" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B238" t="s">
+        <v>239</v>
+      </c>
+      <c r="C238" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B239" t="s">
+        <v>240</v>
+      </c>
+      <c r="C239" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B240" t="s">
+        <v>241</v>
+      </c>
+      <c r="C240" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="241" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B241" t="s">
+        <v>242</v>
+      </c>
+      <c r="C241" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B242" t="s">
+        <v>243</v>
+      </c>
+      <c r="C242" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B243" t="s">
+        <v>244</v>
+      </c>
+      <c r="C243" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B244" t="s">
+        <v>245</v>
+      </c>
+      <c r="C244" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B245" t="s">
+        <v>246</v>
+      </c>
+      <c r="C245" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="246" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B246" t="s">
+        <v>247</v>
+      </c>
+      <c r="C246" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="247" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B247" t="s">
+        <v>248</v>
+      </c>
+      <c r="C247" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B248" t="s">
+        <v>249</v>
+      </c>
+      <c r="C248" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B249" t="s">
+        <v>250</v>
+      </c>
+      <c r="C249" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>